<commit_message>
Support serverless queue dispatching, session credentials persistence, and 24/7 active window
</commit_message>
<xml_diff>
--- a/colleges_delhi_ncr_google_sheets.xlsx
+++ b/colleges_delhi_ncr_google_sheets.xlsx
@@ -522,13 +522,13 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -618,13 +618,13 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="39" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
@@ -944,7 +944,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Amity University, Noida</t>
+          <t>Alpha Engineering College</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -954,36 +954,28 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Noida Sector 125</t>
+          <t>Rohini, Delhi</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Engineering &amp; Management</t>
-        </is>
-      </c>
+      <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>placements@amity.edu</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Head - Corporate Resource Centre</t>
-        </is>
-      </c>
+          <t>tpo@alpha.edu</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>placement</t>
@@ -992,7 +984,7 @@
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -1007,16 +999,12 @@
           <t>Never</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t>Original company CSV. Email and placement role not yet source-checked.</t>
-        </is>
-      </c>
+      <c r="R5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Apex Institute of Technology</t>
+          <t>Amity University, Noida</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1036,28 +1024,24 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Sector 62, Noida</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Main Campus</t>
-        </is>
-      </c>
+          <t>Noida Sector 125</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Technology</t>
+          <t>Engineering &amp; Management</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>placements@apex.edu.in</t>
+          <t>placements@amity.edu</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Dr. Rajesh Sharma</t>
+          <t>Head - Corporate Resource Centre</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -1065,14 +1049,10 @@
           <t>placement</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>0120-1234567</t>
-        </is>
-      </c>
+      <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>unverified</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -1087,7 +1067,11 @@
           <t>Never</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>Original company CSV. Email and placement role not yet source-checked.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1164,7 +1148,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Bhagwan Parshuram Institute of Technology (BPIT)</t>
+          <t>Beta Institute of Tech</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1174,36 +1158,28 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Delhi (GGSIPU)</t>
+          <t>Sector 62, Noida</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Engineering &amp; MBA</t>
-        </is>
-      </c>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>tpo@bpitindia.com</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>Training &amp; Placement Officer</t>
-        </is>
-      </c>
+          <t>placement@beta.ac.in</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr">
         <is>
           <t>placement</t>
@@ -1212,7 +1188,7 @@
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -1227,16 +1203,12 @@
           <t>Never</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>Original company CSV. Email and placement role not yet source-checked.</t>
-        </is>
-      </c>
+      <c r="R8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Bharati Vidyapeeth's College of Engineering (BVCOE)</t>
+          <t>Bhagwan Parshuram Institute of Technology (BPIT)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1262,18 +1234,18 @@
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Tech</t>
+          <t>Engineering &amp; MBA</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>tpo.bvcoe@bharatividyapeeth.edu</t>
+          <t>tpo@bpitindia.com</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Placement Officer</t>
+          <t>Training &amp; Placement Officer</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1308,7 +1280,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Delhi Technological University (DTU)</t>
+          <t>Bharati Vidyapeeth's College of Engineering (BVCOE)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1328,7 +1300,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Delhi (GGSIPU)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
@@ -1340,12 +1312,12 @@
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>placements@dtu.ac.in</t>
+          <t>tpo.bvcoe@bharatividyapeeth.edu</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Head - Training and Placement Department</t>
+          <t>Placement Officer</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1380,7 +1352,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Galgotias College of Engineering and Technology (GCET)</t>
+          <t>Delhi Technological University (DTU)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1390,34 +1362,34 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; MCA</t>
+          <t>Engineering &amp; Tech</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>tpo@galgotiacollege.edu</t>
+          <t>placements@dtu.ac.in</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Training and Placement Officer</t>
+          <t>Head - Training and Placement Department</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1452,7 +1424,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Galgotias University</t>
+          <t>Galgotias College of Engineering and Technology (GCET)</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1478,18 +1450,18 @@
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Engineering, Management &amp; Medical</t>
+          <t>Engineering &amp; MCA</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>placements@galgotiasuniversity.edu.in</t>
+          <t>tpo@galgotiacollege.edu</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Director - Career Planning &amp; Development</t>
+          <t>Training and Placement Officer</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
@@ -1524,7 +1496,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha University (GBU)</t>
+          <t>Galgotias University</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1550,18 +1522,18 @@
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Management</t>
+          <t>Engineering, Management &amp; Medical</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>crc@gbu.ac.in</t>
+          <t>placements@galgotiasuniversity.edu.in</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Head - Corporate Relations Cell</t>
+          <t>Director - Career Planning &amp; Development</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1596,7 +1568,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>GL Bajaj Institute of Technology and Management</t>
+          <t>Gamma University</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1606,36 +1578,28 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Sohna Road</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Engineering &amp; Management</t>
-        </is>
-      </c>
+      <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>tpo@glbitm.ac.in</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Head - Training &amp; Placement Cell</t>
-        </is>
-      </c>
+          <t>corporate@gamma.edu</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr">
         <is>
           <t>placement</t>
@@ -1644,7 +1608,7 @@
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>unverified</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -1659,16 +1623,12 @@
           <t>Never</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
-        <is>
-          <t>Original company CSV. Email and placement role not yet source-checked.</t>
-        </is>
-      </c>
+      <c r="R14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Guru Gobind Singh Indraprastha University (GGSIPU)</t>
+          <t>Gautam Buddha University (GBU)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1678,34 +1638,34 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Delhi (Dwarka)</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Central University</t>
+          <t>Engineering &amp; Management</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>cpc@ipu.ac.in</t>
+          <t>crc@gbu.ac.in</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Director - Central Placement Cell</t>
+          <t>Head - Corporate Relations Cell</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1740,7 +1700,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>IIMT Group of Colleges</t>
+          <t>GL Bajaj Institute of Technology and Management</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1772,12 +1732,12 @@
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>tpo@iimtindia.net</t>
+          <t>tpo@glbitm.ac.in</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Training &amp; Placement Officer</t>
+          <t>Head - Training &amp; Placement Cell</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -1812,7 +1772,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>IMS Engineering College</t>
+          <t>Guru Gobind Singh Indraprastha University (GGSIPU)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1822,34 +1782,34 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Delhi (Dwarka)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Management</t>
+          <t>Central University</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>tpo@imsec.ac.in</t>
+          <t>cpc@ipu.ac.in</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Head - CRC</t>
+          <t>Director - Central Placement Cell</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -1884,7 +1844,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>IMS Ghaziabad (University Courses Campus)</t>
+          <t>IIMT Group of Colleges</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1894,34 +1854,34 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Management &amp; Computer Science</t>
+          <t>Engineering &amp; Management</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>crc@ims-ghaziabad.ac.in</t>
+          <t>tpo@iimtindia.net</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Head - Corporate Relations</t>
+          <t>Training &amp; Placement Officer</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
@@ -1956,7 +1916,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>ITS Engineering College</t>
+          <t>IMS Engineering College</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1966,17 +1926,17 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
@@ -1988,7 +1948,7 @@
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>crc.ec@its.edu.in</t>
+          <t>tpo@imsec.ac.in</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2028,7 +1988,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Jaypee Institute of Information Technology (JIIT)</t>
+          <t>IMS Ghaziabad (University Courses Campus)</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2038,34 +1998,34 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Noida</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Noida Sector 62</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; IT</t>
+          <t>Management &amp; Computer Science</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>placement@jiit.ac.in</t>
+          <t>crc@ims-ghaziabad.ac.in</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Training &amp; Placement Officer</t>
+          <t>Head - Corporate Relations</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
@@ -2100,7 +2060,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>JSS Academy of Technical Education (JSSATE)</t>
+          <t>ITS Engineering College</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -2110,7 +2070,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Noida</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -2120,7 +2080,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Noida Sector 62</t>
+          <t>Greater Noida</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
@@ -2132,12 +2092,12 @@
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>tpo@jssaten.ac.in</t>
+          <t>crc.ec@its.edu.in</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Head - Training and Placement</t>
+          <t>Head - CRC</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -2172,7 +2132,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>KIET Group of Institutions</t>
+          <t>Jaypee Institute of Information Technology (JIIT)</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2182,34 +2142,34 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Ghaziabad</t>
+          <t>Noida Sector 62</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Pharmacy</t>
+          <t>Engineering &amp; IT</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>crpc@kiet.edu</t>
+          <t>placement@jiit.ac.in</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Dean - Corporate Relations</t>
+          <t>Training &amp; Placement Officer</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -2244,7 +2204,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Maharaja Agrasen Institute of Technology (MAIT)</t>
+          <t>JSS Academy of Technical Education (JSSATE)</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -2254,17 +2214,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Gautam Buddha Nagar</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Delhi (GGSIPU)</t>
+          <t>Noida Sector 62</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
@@ -2276,12 +2236,12 @@
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>placements@mait.ac.in</t>
+          <t>tpo@jssaten.ac.in</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>T&amp;P Cell Head</t>
+          <t>Head - Training and Placement</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -2316,7 +2276,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Netaji Subhas University of Technology (NSUT)</t>
+          <t>KIET Group of Institutions</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2326,34 +2286,34 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Ghaziabad</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Tech</t>
+          <t>Engineering &amp; Pharmacy</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>placements@nsut.ac.in</t>
+          <t>crpc@kiet.edu</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Head - Training &amp; Placement Cell</t>
+          <t>Dean - Corporate Relations</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -2388,7 +2348,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Noida Institute of Engineering and Technology (NIET)</t>
+          <t>Maharaja Agrasen Institute of Technology (MAIT)</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -2398,34 +2358,34 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi (GGSIPU)</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Pharmacy</t>
+          <t>Engineering &amp; Management</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>placements@niet.co.in</t>
+          <t>placements@mait.ac.in</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Director - Corporate Relations</t>
+          <t>T&amp;P Cell Head</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -2460,7 +2420,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Sharda University</t>
+          <t>Netaji Subhas University of Technology (NSUT)</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2470,34 +2430,34 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Gautam Buddha Nagar</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Greater Noida</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Engineering, Management &amp; Healthcare</t>
+          <t>Engineering &amp; Tech</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>placement@sharda.ac.in</t>
+          <t>placements@nsut.ac.in</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Head - Training and Placement Cell</t>
+          <t>Head - Training &amp; Placement Cell</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -2532,7 +2492,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Shiv Nadar University (SNU)</t>
+          <t>Noida Institute of Engineering and Technology (NIET)</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2558,18 +2518,18 @@
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Engineering &amp; Science</t>
+          <t>Engineering &amp; Pharmacy</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>careerdevelopment@snu.edu.in</t>
+          <t>placements@niet.co.in</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Career Development Center</t>
+          <t>Director - Corporate Relations</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
@@ -2596,6 +2556,150 @@
         </is>
       </c>
       <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>Original company CSV. Email and placement role not yet source-checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Sharda University</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Colleges</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Gautam Buddha Nagar</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Engineering, Management &amp; Healthcare</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>placement@sharda.ac.in</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Head - Training and Placement Cell</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr"/>
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>Original company CSV. Email and placement role not yet source-checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Shiv Nadar University (SNU)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Colleges</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Gautam Buddha Nagar</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Greater Noida</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Science</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>careerdevelopment@snu.edu.in</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Career Development Center</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>placement</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>Not Contacted</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr"/>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Never</t>
+        </is>
+      </c>
+      <c r="R29" s="4" t="inlineStr">
         <is>
           <t>Original company CSV. Email and placement role not yet source-checked.</t>
         </is>

</xml_diff>